<commit_message>
feat: import full-history opening balances
</commit_message>
<xml_diff>
--- a/fixtures/sanitized/m5/full-import-history.xlsx
+++ b/fixtures/sanitized/m5/full-import-history.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="154">
   <si>
     <t>template_version</t>
   </si>
@@ -234,6 +234,24 @@
     <t>fee_fx_override_reason</t>
   </si>
   <si>
+    <t>OpeningBalance</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Synthetic Merchant</t>
+  </si>
+  <si>
+    <t>Synthetic row</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Synthetic</t>
+  </si>
+  <si>
     <t>2026-01-01</t>
   </si>
   <si>
@@ -243,18 +261,6 @@
     <t>1000</t>
   </si>
   <si>
-    <t>Synthetic Merchant</t>
-  </si>
-  <si>
-    <t>Synthetic row</t>
-  </si>
-  <si>
-    <t>ok</t>
-  </si>
-  <si>
-    <t>Synthetic</t>
-  </si>
-  <si>
     <t>2026-03-05</t>
   </si>
   <si>
@@ -447,6 +453,9 @@
     <t>events</t>
   </si>
   <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>valuation</t>
   </si>
   <si>
@@ -456,7 +465,7 @@
     <t>valued_net_assets</t>
   </si>
   <si>
-    <t>7140</t>
+    <t>7840</t>
   </si>
   <si>
     <t>start_date</t>
@@ -852,13 +861,13 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
@@ -866,13 +875,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -893,16 +902,16 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E1" t="s">
         <v>45</v>
@@ -913,13 +922,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -952,28 +961,28 @@
         <v>51</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L1" t="s">
         <v>58</v>
@@ -982,10 +991,10 @@
         <v>54</v>
       </c>
       <c r="N1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P1" t="s">
         <v>62</v>
@@ -999,28 +1008,28 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s">
         <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F2" t="s">
         <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I2" t="s">
         <v>38</v>
@@ -1032,30 +1041,30 @@
         <v>47</v>
       </c>
       <c r="R2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:18">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
         <v>23</v>
       </c>
       <c r="J3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K3" t="s">
         <v>38</v>
@@ -1066,19 +1075,19 @@
     </row>
     <row r="4" spans="1:18">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B4" t="s">
         <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F4" t="s">
         <v>23</v>
@@ -1087,7 +1096,7 @@
         <v>42</v>
       </c>
       <c r="N4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1102,51 +1111,51 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H1" t="s">
         <v>18</v>
       </c>
       <c r="I1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
         <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G2" t="s">
         <v>42</v>
@@ -1155,7 +1164,7 @@
         <v>26</v>
       </c>
       <c r="I2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1170,30 +1179,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B1" t="s">
         <v>6</v>
       </c>
       <c r="C1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
@@ -1201,13 +1210,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D3" t="s">
         <v>38</v>
@@ -1215,13 +1224,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" t="s">
         <v>135</v>
-      </c>
-      <c r="C4" t="s">
-        <v>133</v>
       </c>
       <c r="D4" t="s">
         <v>38</v>
@@ -1229,13 +1238,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D5" t="s">
         <v>38</v>
@@ -1243,13 +1252,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D6" t="s">
         <v>42</v>
@@ -1260,10 +1269,10 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D7" t="s">
         <v>38</v>
@@ -1271,33 +1280,33 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B9" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D9" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1312,36 +1321,36 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E2" t="s">
         <v>38</v>
@@ -1583,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1650,72 +1659,104 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
         <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
         <v>23</v>
       </c>
-      <c r="E2" t="s">
-        <v>34</v>
-      </c>
       <c r="F2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" t="s">
         <v>70</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>71</v>
-      </c>
-      <c r="H2" t="s">
-        <v>72</v>
       </c>
       <c r="I2" t="s">
         <v>37</v>
       </c>
       <c r="M2" t="s">
+        <v>72</v>
+      </c>
+      <c r="N2" t="s">
         <v>73</v>
-      </c>
-      <c r="N2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" t="s">
         <v>71</v>
-      </c>
-      <c r="H3" t="s">
-        <v>72</v>
       </c>
       <c r="I3" t="s">
         <v>37</v>
       </c>
       <c r="M3" t="s">
+        <v>72</v>
+      </c>
+      <c r="N3" t="s">
         <v>73</v>
       </c>
-      <c r="N3" t="s">
-        <v>74</v>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>72</v>
+      </c>
+      <c r="N4" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1736,10 +1777,10 @@
         <v>50</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E1" t="s">
         <v>54</v>
@@ -1775,16 +1816,16 @@
         <v>50</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G1" t="s">
         <v>57</v>
@@ -1796,22 +1837,22 @@
         <v>56</v>
       </c>
       <c r="J1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="N1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="P1" t="s">
         <v>65</v>
@@ -1841,13 +1882,13 @@
         <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
         <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F1" t="s">
         <v>10</v>
@@ -1861,7 +1902,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -1870,10 +1911,10 @@
         <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F2" t="s">
         <v>15</v>

</xml_diff>